<commit_message>
Unificar saludo de correos a Estimado Cliente
</commit_message>
<xml_diff>
--- a/files/asientos.xlsx
+++ b/files/asientos.xlsx
@@ -1240,6 +1240,11 @@
       <c r="J18" t="n">
         <v>2401</v>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1455,6 +1460,11 @@
       <c r="J23" t="n">
         <v>2401</v>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>CONSORCIO ELECTRICO DE VILLACURI S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1646,6 +1656,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O27" t="n">
         <v>7000002213</v>
       </c>
@@ -2158,6 +2173,11 @@
       <c r="J38" t="n">
         <v>2401</v>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O38" t="n">
         <v>7000002212</v>
       </c>
@@ -2726,7 +2746,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>TRABAJADOR-72714263</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2898,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16733606</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2947,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40554960</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2996,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16736597</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3148,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17450838</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3175,6 +3195,11 @@
           <t>PAGO PROVEEDORES RIPLE</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>TIENDAS POR DEPARTAMENTO RIPLEY S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3270,7 +3295,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16637191</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3393,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16562947</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3442,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17450805</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3491,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17624824</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3540,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16689857</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3589,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16796766</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3677,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761556</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -4153,6 +4178,11 @@
           <t>Pago Fact.203712041620</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>COMPANIA ELECTRICA EL PLATANAL S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4379,6 +4409,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O86" t="n">
         <v>7000002099</v>
       </c>
@@ -4759,6 +4794,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>ON EMPRESAS S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5249,6 +5289,11 @@
       <c r="J105" t="n">
         <v>2401</v>
       </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O105" t="n">
         <v>7000002097</v>
       </c>
@@ -5545,7 +5590,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761208</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O111" t="n">
@@ -5797,6 +5842,11 @@
       <c r="J116" t="n">
         <v>2401</v>
       </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5985,7 +6035,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17625165</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O120" t="n">
@@ -6221,7 +6271,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16759780</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O125" t="n">
@@ -6379,7 +6429,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6672,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>TRABAJADOR-26737638</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O133" t="n">
@@ -6674,7 +6724,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O134" t="n">
@@ -6726,7 +6776,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45385378</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O135" t="n">
@@ -8188,6 +8238,11 @@
       <c r="J167" t="n">
         <v>2401</v>
       </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>VIETTEL PERU S.A.C - CAJ</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8232,6 +8287,11 @@
           <t>Pago0002301550-2026-FE</t>
         </is>
       </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>FENIX POWER PERU S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8474,6 +8534,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O173" t="n">
         <v>7000002086</v>
       </c>
@@ -8890,6 +8955,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>ALDEAS INFANTILES SOS PERU - ASOCIACION NACIONAL</t>
+        </is>
+      </c>
       <c r="O182" t="n">
         <v>7000002143</v>
       </c>
@@ -8932,6 +9002,11 @@
       <c r="J183" t="n">
         <v>2401</v>
       </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O183" t="n">
         <v>7000002085</v>
       </c>
@@ -8974,6 +9049,11 @@
       <c r="J184" t="n">
         <v>2401</v>
       </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>REPRESENT.Y SERVICIOS - INGENIEROS SRL</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9208,7 +9288,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40042745</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O189" t="n">
@@ -9414,6 +9494,11 @@
       <c r="J193" t="n">
         <v>2401</v>
       </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>REPRESENT.Y SERVICIOS - INGENIEROS SRL</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9695,7 +9780,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16729500</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O199" t="n">
@@ -9942,7 +10027,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16753094</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O204" t="n">
@@ -10098,7 +10183,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O207" t="n">
@@ -10333,7 +10418,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16683457</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O212" t="n">
@@ -10855,7 +10940,7 @@
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>TRABAJADOR-41756285</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O223" t="n">
@@ -11041,6 +11126,11 @@
       <c r="J227" t="n">
         <v>2401</v>
       </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>EGEMSA</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -12041,6 +12131,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O251" t="n">
         <v>7000002015</v>
       </c>
@@ -12613,6 +12708,11 @@
       <c r="J263" t="n">
         <v>2401</v>
       </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O263" t="n">
         <v>7000002016</v>
       </c>
@@ -13073,6 +13173,11 @@
       <c r="J273" t="n">
         <v>2401</v>
       </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>DIAR INGENIEROS S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -13119,7 +13224,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>TRABAJADOR-7531871</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O274" t="n">
@@ -13347,7 +13452,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16754694</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -13554,7 +13659,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16735252</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O283" t="n">
@@ -13606,7 +13711,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16423762</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O284" t="n">
@@ -13827,6 +13932,11 @@
       <c r="J289" t="n">
         <v>2401</v>
       </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>EMPRESA DE GENERACION ELECTRICA DE AREQUIPA S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -13873,7 +13983,7 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16762908</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -16814,6 +16924,11 @@
           <t>0000010041</t>
         </is>
       </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>KONDU S.A.C</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -16858,6 +16973,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>FIDEICOMISO ELECTROPERU</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -16902,6 +17022,11 @@
           <t>0000010041</t>
         </is>
       </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>KALLPA GENERACION SA</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -16941,6 +17066,11 @@
       <c r="J364" t="n">
         <v>2401</v>
       </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
       <c r="O364" t="n">
         <v>7000001902</v>
       </c>
@@ -17025,6 +17155,11 @@
       <c r="J366" t="n">
         <v>2401</v>
       </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>COFIDE FID FISE</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -17262,6 +17397,11 @@
           <t>0000010041</t>
         </is>
       </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>ORAZUL ENERGY PERU SA</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -17410,6 +17550,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O374" t="n">
         <v>7000002001</v>
       </c>
@@ -17969,6 +18114,11 @@
       <c r="J386" t="n">
         <v>2401</v>
       </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
       <c r="O386" t="n">
         <v>7000002066</v>
       </c>
@@ -18011,6 +18161,11 @@
       <c r="J387" t="n">
         <v>2401</v>
       </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -18287,7 +18442,7 @@
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16661452</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -18336,7 +18491,7 @@
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16715161</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -19065,7 +19220,7 @@
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16753094</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O409" t="n">
@@ -19110,6 +19265,11 @@
       <c r="J410" t="n">
         <v>2401</v>
       </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O410" t="n">
         <v>7000001996</v>
       </c>
@@ -19201,6 +19361,11 @@
       <c r="J412" t="n">
         <v>2401</v>
       </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>ENTIDAD PRESTADORA DE SERVICIOS DE SANEA</t>
+        </is>
+      </c>
       <c r="O412" t="n">
         <v>7000002067</v>
       </c>
@@ -19421,7 +19586,7 @@
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16659349</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O416" t="n">
@@ -19473,7 +19638,7 @@
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17631880</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O417" t="n">
@@ -22590,7 +22755,7 @@
       </c>
       <c r="M483" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17624824</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O483" t="n">
@@ -22736,7 +22901,7 @@
       </c>
       <c r="M486" t="inlineStr">
         <is>
-          <t>TRABAJADOR-17617984</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O486" t="n">
@@ -22788,7 +22953,7 @@
       </c>
       <c r="M487" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16715161</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O487" t="n">
@@ -24056,7 +24221,7 @@
       </c>
       <c r="M514" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -24105,7 +24270,7 @@
       </c>
       <c r="M515" t="inlineStr">
         <is>
-          <t>TRABAJADOR-40179551</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -24152,6 +24317,11 @@
           <t>Ref 20103117560-01-F06</t>
         </is>
       </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>VARI ENERGIA SAC</t>
+        </is>
+      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -25366,6 +25536,11 @@
           <t>S017603022026</t>
         </is>
       </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>LUZ DEL SUR S.A.A.</t>
+        </is>
+      </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -25603,6 +25778,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O550" t="n">
         <v>7000001737</v>
       </c>
@@ -26162,6 +26342,11 @@
       <c r="J562" t="n">
         <v>2401</v>
       </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O562" t="n">
         <v>7000001735</v>
       </c>
@@ -26268,7 +26453,7 @@
       </c>
       <c r="M564" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16754694</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -26367,6 +26552,11 @@
       <c r="J566" t="n">
         <v>2401</v>
       </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>VIETTEL PERU S.A.C - CAJ</t>
+        </is>
+      </c>
       <c r="O566" t="n">
         <v>7000002106</v>
       </c>
@@ -26565,6 +26755,11 @@
       <c r="J570" t="n">
         <v>2401</v>
       </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>VIETTEL PERU S.A.C - CAJ</t>
+        </is>
+      </c>
       <c r="O570" t="n">
         <v>7000002105</v>
       </c>
@@ -26715,7 +26910,7 @@
       </c>
       <c r="M573" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16687406</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O573" t="n">
@@ -26804,6 +26999,11 @@
       <c r="J575" t="n">
         <v>2401</v>
       </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>TERMOSELVA S.R.L.</t>
+        </is>
+      </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
@@ -26848,6 +27048,11 @@
           <t>S018104022026</t>
         </is>
       </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>INLAND ENERGY SAC</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -26892,6 +27097,11 @@
           <t>01-F061-00020521</t>
         </is>
       </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>INVERSIONES SHAQSHA S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -27986,6 +28196,11 @@
           <t>01-F061-00020467</t>
         </is>
       </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>STATKRAFT PERU SA</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -28220,6 +28435,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O608" t="n">
         <v>7000001608</v>
       </c>
@@ -28316,6 +28536,11 @@
           <t>Pago beneficiario</t>
         </is>
       </c>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>ELECTRO DUNAS S.A.A.</t>
+        </is>
+      </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -28908,6 +29133,11 @@
       <c r="J622" t="n">
         <v>2401</v>
       </c>
+      <c r="L622" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O622" t="n">
         <v>7000001606</v>
       </c>
@@ -29254,7 +29484,7 @@
       </c>
       <c r="M629" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16683457</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O629" t="n">
@@ -29514,7 +29744,7 @@
       </c>
       <c r="M634" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -29563,7 +29793,7 @@
       </c>
       <c r="M635" t="inlineStr">
         <is>
-          <t>TRABAJADOR-72644789</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -29610,6 +29840,11 @@
           <t>Pago Fact.20494</t>
         </is>
       </c>
+      <c r="L636" t="inlineStr">
+        <is>
+          <t>TERMOCHILCA S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -29703,6 +29938,11 @@
           <t>Pago Fact.20485</t>
         </is>
       </c>
+      <c r="L638" t="inlineStr">
+        <is>
+          <t>COMPANIA ELECTRICA EL PLATANAL S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
@@ -29747,6 +29987,11 @@
           <t>Pago Fact.20505</t>
         </is>
       </c>
+      <c r="L639" t="inlineStr">
+        <is>
+          <t>CELEPSA RENOVABLES SRL</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -30749,6 +30994,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
       <c r="O662" t="n">
         <v>6900000034</v>
       </c>
@@ -31246,6 +31496,11 @@
       <c r="J672" t="n">
         <v>2401</v>
       </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
       <c r="O672" t="n">
         <v>6900000023</v>
       </c>
@@ -31485,7 +31740,7 @@
       </c>
       <c r="M677" t="inlineStr">
         <is>
-          <t>TRABAJADOR-43157511</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O677" t="n">
@@ -31916,7 +32171,7 @@
       </c>
       <c r="M686" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16733606</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O686" t="n">
@@ -32015,7 +32270,7 @@
       </c>
       <c r="M688" t="inlineStr">
         <is>
-          <t>TRABAJADOR-41652040</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O688" t="n">
@@ -32453,7 +32708,7 @@
       </c>
       <c r="M697" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16702986</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O697" t="n">
@@ -32505,7 +32760,7 @@
       </c>
       <c r="M698" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16590196</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -33165,7 +33420,7 @@
       </c>
       <c r="M712" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16722058</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O712" t="n">
@@ -33215,6 +33470,11 @@
           <t>Pago0002300998-2026-FE</t>
         </is>
       </c>
+      <c r="L713" t="inlineStr">
+        <is>
+          <t>FENIX POWER PERU S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
@@ -33357,7 +33617,7 @@
       </c>
       <c r="M716" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16423762</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -33406,7 +33666,7 @@
       </c>
       <c r="M717" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16722058</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O717" t="n">
@@ -33451,6 +33711,11 @@
       <c r="J718" t="n">
         <v>2401</v>
       </c>
+      <c r="L718" t="inlineStr">
+        <is>
+          <t>EMPRESA DE GENERACION ELECTRICA SAN GABAN S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" t="inlineStr">
@@ -34437,6 +34702,11 @@
           <t>Referencia Beneficiari</t>
         </is>
       </c>
+      <c r="L741" t="inlineStr">
+        <is>
+          <t>WESTERN UNION PERU S.A.</t>
+        </is>
+      </c>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -35432,7 +35702,7 @@
       </c>
       <c r="M762" t="inlineStr">
         <is>
-          <t>TRABAJADOR-42853214</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -36101,6 +36371,11 @@
       <c r="J776" t="n">
         <v>2401</v>
       </c>
+      <c r="L776" t="inlineStr">
+        <is>
+          <t>CAJA MUNICIPAL DE AHORRO Y CREDITO DE AR</t>
+        </is>
+      </c>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr">
@@ -36204,7 +36479,7 @@
       </c>
       <c r="M778" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16729500</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O778" t="n">
@@ -36459,7 +36734,7 @@
       </c>
       <c r="M783" t="inlineStr">
         <is>
-          <t>TRABAJADOR-16761556</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O783" t="n">
@@ -36553,7 +36828,7 @@
       </c>
       <c r="M785" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O785" t="n">
@@ -36605,7 +36880,7 @@
       </c>
       <c r="M786" t="inlineStr">
         <is>
-          <t>TRABAJADOR-45080863</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O786" t="n">
@@ -36847,7 +37122,7 @@
       </c>
       <c r="M791" t="inlineStr">
         <is>
-          <t>TRABAJADOR-26737638</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O791" t="n">
@@ -37042,6 +37317,11 @@
           <t>PAGO DE PROVEEDORES</t>
         </is>
       </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>FIDEICOMISO ELECTROPERU</t>
+        </is>
+      </c>
     </row>
     <row r="796">
       <c r="A796" t="inlineStr">
@@ -37137,7 +37417,7 @@
       </c>
       <c r="M797" t="inlineStr">
         <is>
-          <t>TRABAJADOR-3701237</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
       <c r="O797" t="n">
@@ -37238,7 +37518,7 @@
       </c>
       <c r="M799" t="inlineStr">
         <is>
-          <t>TRABAJADOR-44465574</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -37380,7 +37660,7 @@
       </c>
       <c r="M802" t="inlineStr">
         <is>
-          <t>TRABAJADOR-71003287</t>
+          <t>TRABAJADOR</t>
         </is>
       </c>
     </row>
@@ -37422,6 +37702,11 @@
       <c r="J803" t="n">
         <v>2401</v>
       </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>HYDRO GLOBAL PERU S.A.C.</t>
+        </is>
+      </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr">
@@ -37464,6 +37749,11 @@
       <c r="K804" t="inlineStr">
         <is>
           <t>Pago beneficiario</t>
+        </is>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>SINDICATO ENERGETICO S.A.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cleanup: remove file-based voucher logic and keep HTML voucher flow
</commit_message>
<xml_diff>
--- a/files/asientos.xlsx
+++ b/files/asientos.xlsx
@@ -2746,7 +2746,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-72714263</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16733606</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-40554960</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16736597</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17450838</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16637191</t>
         </is>
       </c>
     </row>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16562947</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17450805</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17624824</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16689857</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16796766</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16761556</t>
         </is>
       </c>
     </row>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16761208</t>
         </is>
       </c>
       <c r="O111" t="n">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17625165</t>
         </is>
       </c>
       <c r="O120" t="n">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16759780</t>
         </is>
       </c>
       <c r="O125" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-43157511</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-26737638</t>
         </is>
       </c>
       <c r="O133" t="n">
@@ -6724,7 +6724,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-40179551</t>
         </is>
       </c>
       <c r="O134" t="n">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-45385378</t>
         </is>
       </c>
       <c r="O135" t="n">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-40042745</t>
         </is>
       </c>
       <c r="O189" t="n">
@@ -9780,7 +9780,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16729500</t>
         </is>
       </c>
       <c r="O199" t="n">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16753094</t>
         </is>
       </c>
       <c r="O204" t="n">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-43157511</t>
         </is>
       </c>
       <c r="O207" t="n">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16683457</t>
         </is>
       </c>
       <c r="O212" t="n">
@@ -10940,7 +10940,7 @@
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-41756285</t>
         </is>
       </c>
       <c r="O223" t="n">
@@ -13224,7 +13224,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-7531871</t>
         </is>
       </c>
       <c r="O274" t="n">
@@ -13452,7 +13452,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16754694</t>
         </is>
       </c>
     </row>
@@ -13659,7 +13659,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16735252</t>
         </is>
       </c>
       <c r="O283" t="n">
@@ -13711,7 +13711,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16423762</t>
         </is>
       </c>
       <c r="O284" t="n">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16762908</t>
         </is>
       </c>
     </row>
@@ -18442,7 +18442,7 @@
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16661452</t>
         </is>
       </c>
     </row>
@@ -18491,7 +18491,7 @@
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16715161</t>
         </is>
       </c>
     </row>
@@ -19220,7 +19220,7 @@
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16753094</t>
         </is>
       </c>
       <c r="O409" t="n">
@@ -19586,7 +19586,7 @@
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16659349</t>
         </is>
       </c>
       <c r="O416" t="n">
@@ -19638,7 +19638,7 @@
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17631880</t>
         </is>
       </c>
       <c r="O417" t="n">
@@ -22755,7 +22755,7 @@
       </c>
       <c r="M483" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17624824</t>
         </is>
       </c>
       <c r="O483" t="n">
@@ -22901,7 +22901,7 @@
       </c>
       <c r="M486" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-17617984</t>
         </is>
       </c>
       <c r="O486" t="n">
@@ -22953,7 +22953,7 @@
       </c>
       <c r="M487" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16715161</t>
         </is>
       </c>
       <c r="O487" t="n">
@@ -24221,7 +24221,7 @@
       </c>
       <c r="M514" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-40179551</t>
         </is>
       </c>
     </row>
@@ -24270,7 +24270,7 @@
       </c>
       <c r="M515" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-40179551</t>
         </is>
       </c>
     </row>
@@ -26453,7 +26453,7 @@
       </c>
       <c r="M564" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16754694</t>
         </is>
       </c>
     </row>
@@ -26910,7 +26910,7 @@
       </c>
       <c r="M573" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16687406</t>
         </is>
       </c>
       <c r="O573" t="n">
@@ -29484,7 +29484,7 @@
       </c>
       <c r="M629" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16683457</t>
         </is>
       </c>
       <c r="O629" t="n">
@@ -29744,7 +29744,7 @@
       </c>
       <c r="M634" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-45080863</t>
         </is>
       </c>
     </row>
@@ -29793,7 +29793,7 @@
       </c>
       <c r="M635" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-72644789</t>
         </is>
       </c>
     </row>
@@ -31740,7 +31740,7 @@
       </c>
       <c r="M677" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-43157511</t>
         </is>
       </c>
       <c r="O677" t="n">
@@ -32171,7 +32171,7 @@
       </c>
       <c r="M686" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16733606</t>
         </is>
       </c>
       <c r="O686" t="n">
@@ -32270,7 +32270,7 @@
       </c>
       <c r="M688" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-41652040</t>
         </is>
       </c>
       <c r="O688" t="n">
@@ -32708,7 +32708,7 @@
       </c>
       <c r="M697" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16702986</t>
         </is>
       </c>
       <c r="O697" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="M698" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16590196</t>
         </is>
       </c>
     </row>
@@ -33420,7 +33420,7 @@
       </c>
       <c r="M712" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16722058</t>
         </is>
       </c>
       <c r="O712" t="n">
@@ -33617,7 +33617,7 @@
       </c>
       <c r="M716" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16423762</t>
         </is>
       </c>
     </row>
@@ -33666,7 +33666,7 @@
       </c>
       <c r="M717" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16722058</t>
         </is>
       </c>
       <c r="O717" t="n">
@@ -35702,7 +35702,7 @@
       </c>
       <c r="M762" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-42853214</t>
         </is>
       </c>
     </row>
@@ -36479,7 +36479,7 @@
       </c>
       <c r="M778" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16729500</t>
         </is>
       </c>
       <c r="O778" t="n">
@@ -36734,7 +36734,7 @@
       </c>
       <c r="M783" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-16761556</t>
         </is>
       </c>
       <c r="O783" t="n">
@@ -36828,7 +36828,7 @@
       </c>
       <c r="M785" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-45080863</t>
         </is>
       </c>
       <c r="O785" t="n">
@@ -36880,7 +36880,7 @@
       </c>
       <c r="M786" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-45080863</t>
         </is>
       </c>
       <c r="O786" t="n">
@@ -37122,7 +37122,7 @@
       </c>
       <c r="M791" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-26737638</t>
         </is>
       </c>
       <c r="O791" t="n">
@@ -37417,7 +37417,7 @@
       </c>
       <c r="M797" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-3701237</t>
         </is>
       </c>
       <c r="O797" t="n">
@@ -37518,7 +37518,7 @@
       </c>
       <c r="M799" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-44465574</t>
         </is>
       </c>
     </row>
@@ -37660,7 +37660,7 @@
       </c>
       <c r="M802" t="inlineStr">
         <is>
-          <t>TRABAJADOR</t>
+          <t>TRABAJADOR-71003287</t>
         </is>
       </c>
     </row>

</xml_diff>